<commit_message>
Photo rename and put my own excel.
</commit_message>
<xml_diff>
--- a/Ewing/8-26 Ewing Gallery Template.xlsx
+++ b/Ewing/8-26 Ewing Gallery Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveutk-my.sharepoint.com/personal/coneil2_vols_utk_edu/Documents/UT Files/Semester 8/Digital Humanities/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Computer Files\UTK\semester 8 Local\DH_200\Ewing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="11_EE22872F66CAC18352571B75917E9B827B1F9662" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42BE55A6-C480-4FCF-96B5-A2117019E065}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CC5804-DD2E-4817-8B0E-1886CAEFAF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-78" yWindow="0" windowWidth="11676" windowHeight="13758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -401,52 +401,6 @@
   <dxfs count="13">
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FF000000"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF000000"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -723,25 +677,71 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
         <bottom style="thin">
           <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
       <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color rgb="FF000000"/>
         </left>
         <right style="thin">
           <color rgb="FF000000"/>
         </right>
-        <top style="thin">
-          <color rgb="FF000000"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF000000"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -764,17 +764,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B10A5F4-96B6-470D-A08A-B619DEDD60F6}" name="Table1" displayName="Table1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7B10A5F4-96B6-470D-A08A-B619DEDD60F6}" name="Table1" displayName="Table1" ref="A1:H8" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="A1:H8" xr:uid="{7B10A5F4-96B6-470D-A08A-B619DEDD60F6}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{AA499410-60D4-4F94-A353-3FB4225FD7F2}" name="Identifier" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{0A425A9C-AB0A-4E77-811D-99AD440C2DED}" name="Title" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{42A3AE92-CED7-4168-AF14-2D637FC1A727}" name="Creator" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{624F367A-7200-4051-850C-9B07B1A66295}" name="Date" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{F79A44D1-A4AA-4BBB-A418-1E9DBBB4D7DA}" name="Extent" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{3E393DC0-0652-4E74-B952-566EB74175AB}" name="Type" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{6ECDAA30-D61E-480F-915A-67041F72BEB1}" name="Rights" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{3FEADD0E-1ADB-4A2E-AF56-0EBA6CE9DBC2}" name="Description" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{AA499410-60D4-4F94-A353-3FB4225FD7F2}" name="Identifier" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{0A425A9C-AB0A-4E77-811D-99AD440C2DED}" name="Title" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{42A3AE92-CED7-4168-AF14-2D637FC1A727}" name="Creator" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{624F367A-7200-4051-850C-9B07B1A66295}" name="Date" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{F79A44D1-A4AA-4BBB-A418-1E9DBBB4D7DA}" name="Extent" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{3E393DC0-0652-4E74-B952-566EB74175AB}" name="Type" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{6ECDAA30-D61E-480F-915A-67041F72BEB1}" name="Rights" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{3FEADD0E-1ADB-4A2E-AF56-0EBA6CE9DBC2}" name="Description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Removed unnecessary photos and named photos to match identifiers.
</commit_message>
<xml_diff>
--- a/Ewing/8-26 Ewing Gallery Template.xlsx
+++ b/Ewing/8-26 Ewing Gallery Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Computer Files\UTK\semester 8 Local\DH_200\Ewing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CC5804-DD2E-4817-8B0E-1886CAEFAF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913C9B31-8149-46CA-90CC-AF1D141B01F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-78" yWindow="0" windowWidth="11676" windowHeight="13758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="9030" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>